<commit_message>
se agregan parámetros como COT, CVC, biometria, topografía corneal
</commit_message>
<xml_diff>
--- a/CodeSystem-fhir4eyes-care-plan-category-cs.xlsx
+++ b/CodeSystem-fhir4eyes-care-plan-category-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-19T17:55:33+00:00</t>
+    <t>2026-08-25T00:41:24+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
correccion UCUM y de auditoria, queda pendiente codificaciones
</commit_message>
<xml_diff>
--- a/CodeSystem-fhir4eyes-care-plan-category-cs.xlsx
+++ b/CodeSystem-fhir4eyes-care-plan-category-cs.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.3.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-25T18:52:20+00:00</t>
+    <t>2026-09-01T17:43:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>